<commit_message>
Add more data analysis steps
- temporality and phases analysis
- outilers per phase and global
- runs stability induction phase and global
- Domain filter
</commit_message>
<xml_diff>
--- a/data/processed/BR_unified.xlsx
+++ b/data/processed/BR_unified.xlsx
@@ -526,7 +526,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2.749802552140058</v>
+        <v>2.773455919377243</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -573,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5587447890900912</v>
+        <v>0.5761038211514041</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -620,7 +620,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.9239575642423211</v>
+        <v>0.9339659565790682</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -667,7 +667,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5564901545988982</v>
+        <v>0.5448632179088977</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -714,7 +714,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.580216202622681</v>
+        <v>0.5941053896405029</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -761,7 +761,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0.3757280680556381</v>
+        <v>0.3752009716951725</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -808,7 +808,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0.310006510940646</v>
+        <v>0.3011422323314344</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -855,7 +855,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2237628998017618</v>
+        <v>0.2266668382158495</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -902,7 +902,7 @@
         <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1385895818962231</v>
+        <v>0.1157151044226831</v>
       </c>
       <c r="K10" t="n">
         <v>0.001376808266290465</v>
@@ -949,10 +949,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>0.03314406113118952</v>
+        <v>0.05124568729178621</v>
       </c>
       <c r="K11" t="n">
-        <v>0.005248128631914831</v>
+        <v>0.005347014673413195</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -996,10 +996,10 @@
         <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.001554755612273669</v>
+        <v>0.01552994802001744</v>
       </c>
       <c r="K12" t="n">
-        <v>0.003215476712786089</v>
+        <v>0.003433263702817092</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1043,10 +1043,10 @@
         <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>0.002965110633940322</v>
+        <v>0.01111272035177954</v>
       </c>
       <c r="K13" t="n">
-        <v>0.00235260107410428</v>
+        <v>0.002501813373853206</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1090,10 +1090,10 @@
         <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>0.004335697191142551</v>
+        <v>0.01638222328481504</v>
       </c>
       <c r="K14" t="n">
-        <v>0.003951423107048204</v>
+        <v>0.004230403432222566</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1137,10 +1137,10 @@
         <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.001213154415409489</v>
+        <v>0.02049518673510231</v>
       </c>
       <c r="K15" t="n">
-        <v>0.007970040752835573</v>
+        <v>0.008726908721994532</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1184,10 +1184,10 @@
         <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.009142449702790094</v>
+        <v>0.01800617114323162</v>
       </c>
       <c r="K16" t="n">
-        <v>0.01152022455374614</v>
+        <v>0.0127523478454764</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1231,10 +1231,10 @@
         <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.0198085537789039</v>
+        <v>0.0126065438887305</v>
       </c>
       <c r="K17" t="n">
-        <v>0.01703435291443738</v>
+        <v>0.01899488434764714</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1278,10 +1278,10 @@
         <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.03266072321200861</v>
+        <v>0.004888259032005427</v>
       </c>
       <c r="K18" t="n">
-        <v>0.02421264414383018</v>
+        <v>0.02727652307745363</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1325,7 +1325,7 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>1.596153041014634</v>
+        <v>1.602482652780022</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1372,7 +1372,7 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0.4301381038792196</v>
+        <v>0.4426272648187739</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -1419,7 +1419,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0.7432892008944086</v>
+        <v>0.756254723376248</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -1466,7 +1466,7 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0.7594888229386928</v>
+        <v>0.7698900213863152</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1513,7 +1513,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0.5423237583108305</v>
+        <v>0.5626832806131878</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1560,7 +1560,7 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0.4615939123646602</v>
+        <v>0.4646634541979658</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -1607,7 +1607,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0.4069504894767969</v>
+        <v>0.4033104103533711</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -1654,7 +1654,7 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0.3369991120050032</v>
+        <v>0.3467013121834466</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1701,7 +1701,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0.1840966733843364</v>
+        <v>0.219672158981188</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1748,10 +1748,10 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.03291675983144628</v>
+        <v>-0.01443284036767783</v>
       </c>
       <c r="K28" t="n">
-        <v>0.007156010880774704</v>
+        <v>0.007290654632824422</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -1795,10 +1795,10 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>-0.0319311045757603</v>
+        <v>-0.006875180994091012</v>
       </c>
       <c r="K29" t="n">
-        <v>0.003465432184020094</v>
+        <v>0.00392368046067105</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -1842,10 +1842,10 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>0.01394783095350125</v>
+        <v>0.0303104165440671</v>
       </c>
       <c r="K30" t="n">
-        <v>-0.001028742878460581</v>
+        <v>-0.0007128893230051735</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -1889,10 +1889,10 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>0.04171447757343651</v>
+        <v>0.05136474067558817</v>
       </c>
       <c r="K31" t="n">
-        <v>0.004862391059123365</v>
+        <v>0.005059640365639088</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -1936,10 +1936,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>-0.00335623760467881</v>
+        <v>0.02084190545087272</v>
       </c>
       <c r="K32" t="n">
-        <v>0.02169172511126489</v>
+        <v>0.02271264005016667</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="n">
-        <v>-0.05454882657230439</v>
+        <v>-0.01233085181282021</v>
       </c>
       <c r="K33" t="n">
-        <v>0.03608693764184519</v>
+        <v>0.03930504216182691</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2030,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0.1400585212443084</v>
+        <v>0.1594228201218592</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -2077,7 +2077,7 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>0.1504406135917352</v>
+        <v>0.1725952089156426</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -2124,7 +2124,7 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0.9583070639980839</v>
+        <v>0.9811285228062829</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -2171,7 +2171,7 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>0.9684702023760831</v>
+        <v>0.9899267093627049</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -2218,7 +2218,7 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>1.063680178980069</v>
+        <v>1.082855621846605</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -2265,7 +2265,7 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>1.072802810229522</v>
+        <v>1.088171383794787</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
@@ -2312,7 +2312,7 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>0.7803806609447596</v>
+        <v>0.7909100352265892</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -2359,7 +2359,7 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>0.6515254927485321</v>
+        <v>0.6560246461456857</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2406,7 +2406,7 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>0.5194806225004457</v>
+        <v>0.5347918232820792</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2453,7 +2453,7 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0.5083615890749829</v>
+        <v>0.5110146526712632</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0.4528438569757303</v>
+        <v>0.4391293101724653</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
@@ -2547,7 +2547,7 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>0.448840326957907</v>
+        <v>0.4273545224251219</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2594,7 +2594,7 @@
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>0.4617136245566012</v>
+        <v>0.4357681646776544</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>0.3249548092678733</v>
+        <v>0.301036495744355</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2688,7 +2688,7 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>0.1576627905912129</v>
+        <v>0.1649699199731483</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2735,10 +2735,10 @@
         <v>1</v>
       </c>
       <c r="J49" t="n">
-        <v>0.03445942862343594</v>
+        <v>0.05675187252667677</v>
       </c>
       <c r="K49" t="n">
-        <v>0.003434006470901758</v>
+        <v>0.003501440435677357</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -2782,10 +2782,10 @@
         <v>1</v>
       </c>
       <c r="J50" t="n">
-        <v>0.004493756854510984</v>
+        <v>0.0287712905668219</v>
       </c>
       <c r="K50" t="n">
-        <v>0.001115474778887938</v>
+        <v>0.001247265780681729</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -2829,10 +2829,10 @@
         <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>-0.01083190573773037</v>
+        <v>0.01456591555824649</v>
       </c>
       <c r="K51" t="n">
-        <v>0.0004122625413826415</v>
+        <v>0.0005617989587166143</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -2876,10 +2876,10 @@
         <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>-0.01669185164159171</v>
+        <v>0.00903844662544389</v>
       </c>
       <c r="K52" t="n">
-        <v>0.00122936272601901</v>
+        <v>0.001400303515493451</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -2923,10 +2923,10 @@
         <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>-0.01179733882199922</v>
+        <v>0.01323117077339356</v>
       </c>
       <c r="K53" t="n">
-        <v>0.002471322711471965</v>
+        <v>0.002695343258845363</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -2970,10 +2970,10 @@
         <v>1</v>
       </c>
       <c r="J54" t="n">
-        <v>0.0001302027365206807</v>
+        <v>0.02382402656220278</v>
       </c>
       <c r="K54" t="n">
-        <v>0.002914316351724278</v>
+        <v>0.003184053625464791</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -3017,7 +3017,7 @@
         <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>1.252035652211464</v>
+        <v>1.260880663338122</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
@@ -3064,7 +3064,7 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>0.5336693857802129</v>
+        <v>0.5497032257743698</v>
       </c>
       <c r="K56" t="n">
         <v>0</v>
@@ -3111,7 +3111,7 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>0.9165615261972639</v>
+        <v>0.9383358366299146</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
@@ -3158,7 +3158,7 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>0.9483374194075437</v>
+        <v>0.9708387821298967</v>
       </c>
       <c r="K58" t="n">
         <v>0</v>
@@ -3205,7 +3205,7 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>1.004181549477588</v>
+        <v>1.026168560890297</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
@@ -3252,7 +3252,7 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>0.9299145096452803</v>
+        <v>0.9494605001325969</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
@@ -3299,7 +3299,7 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>0.7950155854527635</v>
+        <v>0.8106051383870165</v>
       </c>
       <c r="K61" t="n">
         <v>0</v>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>0.65638633197089</v>
+        <v>0.6663713662008954</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>0.6205962372214493</v>
+        <v>0.6235689381655682</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -3440,7 +3440,7 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>0.4923992943307707</v>
+        <v>0.4795308183916825</v>
       </c>
       <c r="K64" t="n">
         <v>0</v>
@@ -3487,7 +3487,7 @@
         <v>0</v>
       </c>
       <c r="J65" t="n">
-        <v>0.4961440893002063</v>
+        <v>0.4846308392588772</v>
       </c>
       <c r="K65" t="n">
         <v>0</v>
@@ -3534,7 +3534,7 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>0.4421199921781828</v>
+        <v>0.4228387269587031</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
@@ -3581,7 +3581,7 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>0.3746413719606005</v>
+        <v>0.3556530235268606</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>0.321751087878845</v>
+        <v>0.3136399914492508</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3675,7 +3675,7 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>0.1569547993441058</v>
+        <v>0.1826458572662279</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
@@ -3722,10 +3722,10 @@
         <v>1</v>
       </c>
       <c r="J70" t="n">
-        <v>0.03026252953345812</v>
+        <v>0.05357868236989675</v>
       </c>
       <c r="K70" t="n">
-        <v>0.002501618914682016</v>
+        <v>0.002547837117342036</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -3769,10 +3769,10 @@
         <v>1</v>
       </c>
       <c r="J71" t="n">
-        <v>-0.005282794515586522</v>
+        <v>0.02080165223917927</v>
       </c>
       <c r="K71" t="n">
-        <v>0.001618404975634121</v>
+        <v>0.001724202920283548</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -3816,10 +3816,10 @@
         <v>1</v>
       </c>
       <c r="J72" t="n">
-        <v>-0.01559845820963498</v>
+        <v>0.009331770144835409</v>
       </c>
       <c r="K72" t="n">
-        <v>0.001276514428093743</v>
+        <v>0.001413804742196162</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -3863,10 +3863,10 @@
         <v>1</v>
       </c>
       <c r="J73" t="n">
-        <v>-0.03887226550383004</v>
+        <v>0.01352004232695701</v>
       </c>
       <c r="K73" t="n">
-        <v>0.0004551706917293473</v>
+        <v>0.0007937774562501765</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -3910,10 +3910,10 @@
         <v>1</v>
       </c>
       <c r="J74" t="n">
-        <v>-0.03242257693292625</v>
+        <v>0.03471573864569432</v>
       </c>
       <c r="K74" t="n">
-        <v>-0.0001360954276419427</v>
+        <v>0.0003337613079274545</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
@@ -3957,10 +3957,10 @@
         <v>1</v>
       </c>
       <c r="J75" t="n">
-        <v>0.07003390164242121</v>
+        <v>0.06234991732197818</v>
       </c>
       <c r="K75" t="n">
-        <v>3.563183147987207e-06</v>
+        <v>-4.864082110984936e-05</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -4004,7 +4004,7 @@
         <v>0</v>
       </c>
       <c r="J76" t="n">
-        <v>-0.06293997995203024</v>
+        <v>-0.04912864042823699</v>
       </c>
       <c r="K76" t="n">
         <v>0</v>
@@ -4051,7 +4051,7 @@
         <v>0</v>
       </c>
       <c r="J77" t="n">
-        <v>0.660061240211836</v>
+        <v>0.6724309901233051</v>
       </c>
       <c r="K77" t="n">
         <v>0</v>
@@ -4098,7 +4098,7 @@
         <v>0</v>
       </c>
       <c r="J78" t="n">
-        <v>0.241729975763457</v>
+        <v>0.2530518459903527</v>
       </c>
       <c r="K78" t="n">
         <v>0</v>
@@ -4145,7 +4145,7 @@
         <v>0</v>
       </c>
       <c r="J79" t="n">
-        <v>0.6674175502593021</v>
+        <v>0.677917507436988</v>
       </c>
       <c r="K79" t="n">
         <v>0</v>
@@ -4192,7 +4192,7 @@
         <v>0</v>
       </c>
       <c r="J80" t="n">
-        <v>1.003375812107504</v>
+        <v>1.013252033425614</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -4239,7 +4239,7 @@
         <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>0.9657863432730587</v>
+        <v>0.9707966960530389</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
@@ -4286,7 +4286,7 @@
         <v>0</v>
       </c>
       <c r="J82" t="n">
-        <v>0.6344026016746118</v>
+        <v>0.6576591536422528</v>
       </c>
       <c r="K82" t="n">
         <v>0</v>
@@ -4333,7 +4333,7 @@
         <v>0</v>
       </c>
       <c r="J83" t="n">
-        <v>0.4486410077707111</v>
+        <v>0.4515050098524599</v>
       </c>
       <c r="K83" t="n">
         <v>0</v>
@@ -4380,7 +4380,7 @@
         <v>0</v>
       </c>
       <c r="J84" t="n">
-        <v>0.4285252010816449</v>
+        <v>0.4182805436774139</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
@@ -4427,7 +4427,7 @@
         <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>0.4415451466267334</v>
+        <v>0.4304201468243027</v>
       </c>
       <c r="K85" t="n">
         <v>0</v>
@@ -4474,7 +4474,7 @@
         <v>0</v>
       </c>
       <c r="J86" t="n">
-        <v>0.3321854551088094</v>
+        <v>0.3439991671540097</v>
       </c>
       <c r="K86" t="n">
         <v>0</v>
@@ -4521,7 +4521,7 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>0.1882431313297978</v>
+        <v>0.2230513338285369</v>
       </c>
       <c r="K87" t="n">
         <v>0</v>
@@ -4568,10 +4568,10 @@
         <v>1</v>
       </c>
       <c r="J88" t="n">
-        <v>-0.01105903752040654</v>
+        <v>0.003107749771201265</v>
       </c>
       <c r="K88" t="n">
-        <v>0.001424028212453621</v>
+        <v>0.001445001091803178</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -4615,10 +4615,10 @@
         <v>1</v>
       </c>
       <c r="J89" t="n">
-        <v>-0.006539483595473478</v>
+        <v>0.01118588271009556</v>
       </c>
       <c r="K89" t="n">
-        <v>0.00106644115300713</v>
+        <v>0.001115254858587295</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -4662,10 +4662,10 @@
         <v>1</v>
       </c>
       <c r="J90" t="n">
-        <v>0.01084002481951049</v>
+        <v>0.02295381943578307</v>
       </c>
       <c r="K90" t="n">
-        <v>0.001336243372152687</v>
+        <v>0.001381250583328814</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -4709,10 +4709,10 @@
         <v>1</v>
       </c>
       <c r="J91" t="n">
-        <v>0.01195244639154316</v>
+        <v>0.02163785772681053</v>
       </c>
       <c r="K91" t="n">
-        <v>0.001578296131698036</v>
+        <v>0.001627618614383601</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -4756,10 +4756,10 @@
         <v>1</v>
       </c>
       <c r="J92" t="n">
-        <v>0.01307042927962515</v>
+        <v>0.01988925556441652</v>
       </c>
       <c r="K92" t="n">
-        <v>0.001426203843877773</v>
+        <v>0.001472810368952698</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -4803,10 +4803,10 @@
         <v>1</v>
       </c>
       <c r="J93" t="n">
-        <v>0.01438956766955691</v>
+        <v>0.01810984717688489</v>
       </c>
       <c r="K93" t="n">
-        <v>0.001528634013203251</v>
+        <v>0.001562397105294549</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
@@ -4850,10 +4850,10 @@
         <v>1</v>
       </c>
       <c r="J94" t="n">
-        <v>0.01515811592377075</v>
+        <v>0.01588198484448558</v>
       </c>
       <c r="K94" t="n">
-        <v>0.001733233396809464</v>
+        <v>0.001741902445938169</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -4897,10 +4897,10 @@
         <v>1</v>
       </c>
       <c r="J95" t="n">
-        <v>0.01417944263470053</v>
+        <v>0.01219923945270092</v>
       </c>
       <c r="K95" t="n">
-        <v>0.001616191983667984</v>
+        <v>0.00157908576545168</v>
       </c>
       <c r="L95" t="inlineStr">
         <is>
@@ -4944,10 +4944,10 @@
         <v>1</v>
       </c>
       <c r="J96" t="n">
-        <v>0.01282160128487731</v>
+        <v>0.0109808124754755</v>
       </c>
       <c r="K96" t="n">
-        <v>0.001550652376102339</v>
+        <v>0.001512631426857109</v>
       </c>
       <c r="L96" t="inlineStr">
         <is>
@@ -4991,10 +4991,10 @@
         <v>1</v>
       </c>
       <c r="J97" t="n">
-        <v>0.009618361020492208</v>
+        <v>0.009505450740006317</v>
       </c>
       <c r="K97" t="n">
-        <v>0.001634591627341015</v>
+        <v>0.001631883077251543</v>
       </c>
       <c r="L97" t="inlineStr">
         <is>
@@ -5038,10 +5038,10 @@
         <v>1</v>
       </c>
       <c r="J98" t="n">
-        <v>0.007340807779644879</v>
+        <v>0.008678513615209167</v>
       </c>
       <c r="K98" t="n">
-        <v>0.001554031431258592</v>
+        <v>0.001589163588687227</v>
       </c>
       <c r="L98" t="inlineStr">
         <is>
@@ -5085,10 +5085,10 @@
         <v>1</v>
       </c>
       <c r="J99" t="n">
-        <v>0.004570300067676985</v>
+        <v>0.007554896901701574</v>
       </c>
       <c r="K99" t="n">
-        <v>0.001262930948401204</v>
+        <v>0.001354066490569085</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
@@ -5132,10 +5132,10 @@
         <v>1</v>
       </c>
       <c r="J100" t="n">
-        <v>0.002924878222549816</v>
+        <v>0.006612622589976032</v>
       </c>
       <c r="K100" t="n">
-        <v>0.0009743033269647772</v>
+        <v>0.001096025468330356</v>
       </c>
       <c r="L100" t="inlineStr">
         <is>
@@ -5179,10 +5179,10 @@
         <v>1</v>
       </c>
       <c r="J101" t="n">
-        <v>0.002593429011303724</v>
+        <v>0.005957167974068228</v>
       </c>
       <c r="K101" t="n">
-        <v>0.0008022173042197786</v>
+        <v>0.0009206718114117425</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
@@ -5226,10 +5226,10 @@
         <v>1</v>
       </c>
       <c r="J102" t="n">
-        <v>0.003298904250178337</v>
+        <v>0.005627786225201607</v>
       </c>
       <c r="K102" t="n">
-        <v>0.0005908681981226406</v>
+        <v>0.0006771604428841338</v>
       </c>
       <c r="L102" t="inlineStr">
         <is>
@@ -5273,10 +5273,10 @@
         <v>1</v>
       </c>
       <c r="J103" t="n">
-        <v>0.009943878835155432</v>
+        <v>0.00579003513273569</v>
       </c>
       <c r="K103" t="n">
-        <v>-0.0001299503672002192</v>
+        <v>-0.0002836589519597477</v>
       </c>
       <c r="L103" t="inlineStr">
         <is>
@@ -5320,7 +5320,7 @@
         <v>0</v>
       </c>
       <c r="J104" t="n">
-        <v>2.178501834629867</v>
+        <v>2.183821215881375</v>
       </c>
       <c r="K104" t="n">
         <v>0</v>
@@ -5367,7 +5367,7 @@
         <v>0</v>
       </c>
       <c r="J105" t="n">
-        <v>0.0908049220820258</v>
+        <v>0.1008732325518622</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
@@ -5414,7 +5414,7 @@
         <v>0</v>
       </c>
       <c r="J106" t="n">
-        <v>0.6313800937079562</v>
+        <v>0.6439354103275791</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
@@ -5461,7 +5461,7 @@
         <v>0</v>
       </c>
       <c r="J107" t="n">
-        <v>0.7483768613607478</v>
+        <v>0.7601922994214217</v>
       </c>
       <c r="K107" t="n">
         <v>0</v>
@@ -5508,7 +5508,7 @@
         <v>0</v>
       </c>
       <c r="J108" t="n">
-        <v>0.7249115499885794</v>
+        <v>0.7338823076920771</v>
       </c>
       <c r="K108" t="n">
         <v>0</v>
@@ -5555,7 +5555,7 @@
         <v>0</v>
       </c>
       <c r="J109" t="n">
-        <v>0.5799692397437735</v>
+        <v>0.5805340652232519</v>
       </c>
       <c r="K109" t="n">
         <v>0</v>
@@ -5602,7 +5602,7 @@
         <v>0</v>
       </c>
       <c r="J110" t="n">
-        <v>0.511193033094957</v>
+        <v>0.5233115654531719</v>
       </c>
       <c r="K110" t="n">
         <v>0</v>
@@ -5649,7 +5649,7 @@
         <v>0</v>
       </c>
       <c r="J111" t="n">
-        <v>0.4739678734978481</v>
+        <v>0.4717503638328068</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
@@ -5696,7 +5696,7 @@
         <v>0</v>
       </c>
       <c r="J112" t="n">
-        <v>0.4195607197080667</v>
+        <v>0.4083034595445517</v>
       </c>
       <c r="K112" t="n">
         <v>0</v>
@@ -5743,7 +5743,7 @@
         <v>0</v>
       </c>
       <c r="J113" t="n">
-        <v>0.2928244321080677</v>
+        <v>0.2748618283353326</v>
       </c>
       <c r="K113" t="n">
         <v>0</v>
@@ -5790,7 +5790,7 @@
         <v>0</v>
       </c>
       <c r="J114" t="n">
-        <v>0.2207507909314687</v>
+        <v>0.2071020657085952</v>
       </c>
       <c r="K114" t="n">
         <v>0</v>
@@ -5837,7 +5837,7 @@
         <v>0</v>
       </c>
       <c r="J115" t="n">
-        <v>0.1612251415110586</v>
+        <v>0.1127203646795815</v>
       </c>
       <c r="K115" t="n">
         <v>0.0001175005555978089</v>
@@ -5884,7 +5884,7 @@
         <v>0</v>
       </c>
       <c r="J116" t="n">
-        <v>0.09975983373459374</v>
+        <v>0.06478986818992959</v>
       </c>
       <c r="K116" t="n">
         <v>-0.0004264984994682457</v>
@@ -5931,7 +5931,7 @@
         <v>0</v>
       </c>
       <c r="J117" t="n">
-        <v>0.02836717272179347</v>
+        <v>0.0205872064904903</v>
       </c>
       <c r="K117" t="n">
         <v>0.00164594032461177</v>
@@ -5978,10 +5978,10 @@
         <v>1</v>
       </c>
       <c r="J118" t="n">
-        <v>-0.004713773159018765</v>
+        <v>0.003021746759544639</v>
       </c>
       <c r="K118" t="n">
-        <v>0.003293043171009324</v>
+        <v>0.003312583250983506</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -6025,10 +6025,10 @@
         <v>1</v>
       </c>
       <c r="J119" t="n">
-        <v>-0.009857319918517854</v>
+        <v>0.0019845574521799</v>
       </c>
       <c r="K119" t="n">
-        <v>0.002654629529526851</v>
+        <v>0.002739171059580418</v>
       </c>
       <c r="L119" t="inlineStr">
         <is>
@@ -6072,10 +6072,10 @@
         <v>1</v>
       </c>
       <c r="J120" t="n">
-        <v>0.01023474019624145</v>
+        <v>0.01455809385433574</v>
       </c>
       <c r="K120" t="n">
-        <v>0.001867354862504477</v>
+        <v>0.001911362494183918</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
@@ -6119,10 +6119,10 @@
         <v>1</v>
       </c>
       <c r="J121" t="n">
-        <v>0.01851487470807779</v>
+        <v>0.01884398231195675</v>
       </c>
       <c r="K121" t="n">
-        <v>0.001310895576645335</v>
+        <v>0.001315088996618529</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -6166,10 +6166,10 @@
         <v>1</v>
       </c>
       <c r="J122" t="n">
-        <v>0.01455499479293736</v>
+        <v>0.01453349632246627</v>
       </c>
       <c r="K122" t="n">
-        <v>5.048555143382714e-05</v>
+        <v>5.015906025550427e-05</v>
       </c>
       <c r="L122" t="inlineStr">
         <is>
@@ -6213,10 +6213,10 @@
         <v>1</v>
       </c>
       <c r="J123" t="n">
-        <v>0.01230461527488503</v>
+        <v>0.01248729650410173</v>
       </c>
       <c r="K123" t="n">
-        <v>-0.0001085942815487884</v>
+        <v>-0.0001059684095731</v>
       </c>
       <c r="L123" t="inlineStr">
         <is>
@@ -6260,10 +6260,10 @@
         <v>1</v>
       </c>
       <c r="J124" t="n">
-        <v>0.008742830430075664</v>
+        <v>0.009728281230436566</v>
       </c>
       <c r="K124" t="n">
-        <v>-0.0001788917976299374</v>
+        <v>-0.0001650741561724392</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -6307,10 +6307,10 @@
         <v>1</v>
       </c>
       <c r="J125" t="n">
-        <v>0.006722095899219682</v>
+        <v>0.008310448961339791</v>
       </c>
       <c r="K125" t="n">
-        <v>-0.0002892203566732219</v>
+        <v>-0.0002678445384691147</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -6354,10 +6354,10 @@
         <v>1</v>
       </c>
       <c r="J126" t="n">
-        <v>0.006136984593039796</v>
+        <v>0.00822136698472653</v>
       </c>
       <c r="K126" t="n">
-        <v>-0.0001823462673344268</v>
+        <v>-0.0001556484430730202</v>
       </c>
       <c r="L126" t="inlineStr">
         <is>
@@ -6401,10 +6401,10 @@
         <v>1</v>
       </c>
       <c r="J127" t="n">
-        <v>0.009186539382775555</v>
+        <v>0.01109926627240091</v>
       </c>
       <c r="K127" t="n">
-        <v>-3.677005945695869e-05</v>
+        <v>-1.403233585153209e-05</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -6448,10 +6448,10 @@
         <v>1</v>
       </c>
       <c r="J128" t="n">
-        <v>0.01244683684439359</v>
+        <v>0.01352430234797856</v>
       </c>
       <c r="K128" t="n">
-        <v>0.000282524793518221</v>
+        <v>0.000295096461983429</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
@@ -6495,10 +6495,10 @@
         <v>1</v>
       </c>
       <c r="J129" t="n">
-        <v>0.01343958719248019</v>
+        <v>0.01327491343608372</v>
       </c>
       <c r="K129" t="n">
-        <v>0.0006464557084945431</v>
+        <v>0.0006443471915813714</v>
       </c>
       <c r="L129" t="inlineStr">
         <is>
@@ -6542,10 +6542,10 @@
         <v>1</v>
       </c>
       <c r="J130" t="n">
-        <v>0.004293081030292754</v>
+        <v>-0.001878942565908728</v>
       </c>
       <c r="K130" t="n">
-        <v>0.002725602305221688</v>
+        <v>0.002583354190690231</v>
       </c>
       <c r="L130" t="inlineStr">
         <is>
@@ -6589,7 +6589,7 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>0.2946058237680711</v>
+        <v>0.3059909272768807</v>
       </c>
       <c r="K131" t="n">
         <v>0</v>
@@ -6636,7 +6636,7 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>1.821183849017537</v>
+        <v>1.827355883937059</v>
       </c>
       <c r="K132" t="n">
         <v>0</v>
@@ -6683,7 +6683,7 @@
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>1.104563214631156</v>
+        <v>1.10741244653135</v>
       </c>
       <c r="K133" t="n">
         <v>0</v>
@@ -6730,7 +6730,7 @@
         <v>0</v>
       </c>
       <c r="J134" t="n">
-        <v>0.6375838666016491</v>
+        <v>0.6415666469506192</v>
       </c>
       <c r="K134" t="n">
         <v>0</v>
@@ -6777,7 +6777,7 @@
         <v>0</v>
       </c>
       <c r="J135" t="n">
-        <v>0.3974511847328741</v>
+        <v>0.4219533314783788</v>
       </c>
       <c r="K135" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>0</v>
       </c>
       <c r="J136" t="n">
-        <v>0.4420688113670645</v>
+        <v>0.4562316630032269</v>
       </c>
       <c r="K136" t="n">
         <v>0</v>
@@ -6871,7 +6871,7 @@
         <v>0</v>
       </c>
       <c r="J137" t="n">
-        <v>0.4196598813961614</v>
+        <v>0.4142626004029457</v>
       </c>
       <c r="K137" t="n">
         <v>0</v>
@@ -6918,7 +6918,7 @@
         <v>0</v>
       </c>
       <c r="J138" t="n">
-        <v>0.3995504457429571</v>
+        <v>0.3767908000623271</v>
       </c>
       <c r="K138" t="n">
         <v>0</v>
@@ -6965,7 +6965,7 @@
         <v>0</v>
       </c>
       <c r="J139" t="n">
-        <v>0.3663838906847608</v>
+        <v>0.3433307891312969</v>
       </c>
       <c r="K139" t="n">
         <v>0</v>
@@ -7012,7 +7012,7 @@
         <v>0</v>
       </c>
       <c r="J140" t="n">
-        <v>0.2779366669743506</v>
+        <v>0.2613926852003742</v>
       </c>
       <c r="K140" t="n">
         <v>0</v>
@@ -7059,7 +7059,7 @@
         <v>0</v>
       </c>
       <c r="J141" t="n">
-        <v>0.1514869727740101</v>
+        <v>0.1618913502923609</v>
       </c>
       <c r="K141" t="n">
         <v>0</v>
@@ -7106,10 +7106,10 @@
         <v>1</v>
       </c>
       <c r="J142" t="n">
-        <v>0.04316917227728913</v>
+        <v>0.04917539497438628</v>
       </c>
       <c r="K142" t="n">
-        <v>0.001800169659733942</v>
+        <v>0.001811100575128213</v>
       </c>
       <c r="L142" t="inlineStr">
         <is>
@@ -7153,10 +7153,10 @@
         <v>1</v>
       </c>
       <c r="J143" t="n">
-        <v>-0.0008855981038328187</v>
+        <v>0.01842353278504401</v>
       </c>
       <c r="K143" t="n">
-        <v>0.001258376380076537</v>
+        <v>0.001329836581426537</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -7200,10 +7200,10 @@
         <v>1</v>
       </c>
       <c r="J144" t="n">
-        <v>0.005175259570775335</v>
+        <v>0.01692570749896018</v>
       </c>
       <c r="K144" t="n">
-        <v>0.001259657785815</v>
+        <v>0.001320393462500107</v>
       </c>
       <c r="L144" t="inlineStr">
         <is>
@@ -7247,10 +7247,10 @@
         <v>1</v>
       </c>
       <c r="J145" t="n">
-        <v>0.01115888856801218</v>
+        <v>0.01517253945036008</v>
       </c>
       <c r="K145" t="n">
-        <v>0.0007821358053090313</v>
+        <v>0.0008079556498792349</v>
       </c>
       <c r="L145" t="inlineStr">
         <is>
@@ -7294,10 +7294,10 @@
         <v>1</v>
       </c>
       <c r="J146" t="n">
-        <v>0.01540493515624475</v>
+        <v>0.01329422655362221</v>
       </c>
       <c r="K146" t="n">
-        <v>0.0005318818171413258</v>
+        <v>0.0005147638662777166</v>
       </c>
       <c r="L146" t="inlineStr">
         <is>
@@ -7341,10 +7341,10 @@
         <v>1</v>
       </c>
       <c r="J147" t="n">
-        <v>0.0138063492230678</v>
+        <v>0.01148120226042161</v>
       </c>
       <c r="K147" t="n">
-        <v>0.0001097251705658746</v>
+        <v>8.924070142373759e-05</v>
       </c>
       <c r="L147" t="inlineStr">
         <is>
@@ -7388,10 +7388,10 @@
         <v>1</v>
       </c>
       <c r="J148" t="n">
-        <v>0.01368141066002931</v>
+        <v>0.01162569995638111</v>
       </c>
       <c r="K148" t="n">
-        <v>9.12282651943517e-05</v>
+        <v>7.319109800795945e-05</v>
       </c>
       <c r="L148" t="inlineStr">
         <is>
@@ -7435,10 +7435,10 @@
         <v>1</v>
       </c>
       <c r="J149" t="n">
-        <v>0.01360211626339042</v>
+        <v>0.01200460307202816</v>
       </c>
       <c r="K149" t="n">
-        <v>9.768471711143985e-05</v>
+        <v>8.366395206795795e-05</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -7482,10 +7482,10 @@
         <v>1</v>
       </c>
       <c r="J150" t="n">
-        <v>0.01362496240594237</v>
+        <v>0.01255262555007765</v>
       </c>
       <c r="K150" t="n">
-        <v>0.0001094397707458446</v>
+        <v>9.984344484120283e-05</v>
       </c>
       <c r="L150" t="inlineStr">
         <is>
@@ -7529,10 +7529,10 @@
         <v>1</v>
       </c>
       <c r="J151" t="n">
-        <v>0.01266956348248249</v>
+        <v>0.01238570420736306</v>
       </c>
       <c r="K151" t="n">
-        <v>0.0001879675924097938</v>
+        <v>0.0001854793019686192</v>
       </c>
       <c r="L151" t="inlineStr">
         <is>
@@ -7576,10 +7576,10 @@
         <v>1</v>
       </c>
       <c r="J152" t="n">
-        <v>0.01187306607807426</v>
+        <v>0.01193612546465203</v>
       </c>
       <c r="K152" t="n">
-        <v>0.0003638605861447401</v>
+        <v>0.0003644512203400279</v>
       </c>
       <c r="L152" t="inlineStr">
         <is>
@@ -7623,10 +7623,10 @@
         <v>1</v>
       </c>
       <c r="J153" t="n">
-        <v>0.01069683576452325</v>
+        <v>0.01075248518714547</v>
       </c>
       <c r="K153" t="n">
-        <v>0.0005699014738202645</v>
+        <v>0.000570465953039973</v>
       </c>
       <c r="L153" t="inlineStr">
         <is>
@@ -7670,10 +7670,10 @@
         <v>1</v>
       </c>
       <c r="J154" t="n">
-        <v>0.009566388737215298</v>
+        <v>0.009349867586919757</v>
       </c>
       <c r="K154" t="n">
-        <v>0.0008289778325600097</v>
+        <v>0.0008263887538865186</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -7717,10 +7717,10 @@
         <v>1</v>
       </c>
       <c r="J155" t="n">
-        <v>0.004296075054780506</v>
+        <v>0.0018847027711307</v>
       </c>
       <c r="K155" t="n">
-        <v>0.001798868823778471</v>
+        <v>0.001747875790330702</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Change qP for rP in data analysis
</commit_message>
<xml_diff>
--- a/data/processed/BR_unified.xlsx
+++ b/data/processed/BR_unified.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M155"/>
+  <dimension ref="A1:N155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,10 +486,15 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>rP</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>T_ind</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Run_T</t>
         </is>
@@ -531,12 +536,15 @@
       <c r="K2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -578,12 +586,15 @@
       <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -625,12 +636,15 @@
       <c r="K4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -672,12 +686,15 @@
       <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -719,12 +736,15 @@
       <c r="K6" t="n">
         <v>0</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -766,12 +786,15 @@
       <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -813,12 +836,15 @@
       <c r="K8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -860,12 +886,15 @@
       <c r="K9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -907,12 +936,15 @@
       <c r="K10" t="n">
         <v>0.001376808266290465</v>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="n">
+        <v>0.03176493357227264</v>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -954,12 +986,15 @@
       <c r="K11" t="n">
         <v>0.005347014673413195</v>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L11" t="n">
+        <v>0.128232869757034</v>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -1001,12 +1036,15 @@
       <c r="K12" t="n">
         <v>0.003433263702817092</v>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L12" t="n">
+        <v>0.08485066008390806</v>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -1048,12 +1086,15 @@
       <c r="K13" t="n">
         <v>0.002501813373853206</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L13" t="n">
+        <v>0.06316185264202921</v>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -1095,12 +1136,15 @@
       <c r="K14" t="n">
         <v>0.004230403432222566</v>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L14" t="n">
+        <v>0.1134289611474972</v>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -1142,12 +1186,15 @@
       <c r="K15" t="n">
         <v>0.008726908721994532</v>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L15" t="n">
+        <v>0.2383692782350503</v>
+      </c>
+      <c r="M15" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -1189,12 +1236,15 @@
       <c r="K16" t="n">
         <v>0.0127523478454764</v>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L16" t="n">
+        <v>0.35264796202687</v>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -1236,12 +1286,15 @@
       <c r="K17" t="n">
         <v>0.01899488434764714</v>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="L17" t="n">
+        <v>0.5326029893334924</v>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -1283,12 +1336,15 @@
       <c r="K18" t="n">
         <v>0.02727652307745363</v>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L18" t="n">
+        <v>0.7751403361689226</v>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>BR02_T_28</t>
         </is>
@@ -1330,12 +1386,15 @@
       <c r="K19" t="n">
         <v>0</v>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1377,12 +1436,15 @@
       <c r="K20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1424,12 +1486,15 @@
       <c r="K21" t="n">
         <v>0</v>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1471,12 +1536,15 @@
       <c r="K22" t="n">
         <v>0</v>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1518,12 +1586,15 @@
       <c r="K23" t="n">
         <v>0</v>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1565,12 +1636,15 @@
       <c r="K24" t="n">
         <v>0</v>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1612,12 +1686,15 @@
       <c r="K25" t="n">
         <v>0</v>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1659,12 +1736,15 @@
       <c r="K26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1706,12 +1786,15 @@
       <c r="K27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1753,12 +1836,15 @@
       <c r="K28" t="n">
         <v>0.007290654632824422</v>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L28" t="n">
+        <v>0.196326914041058</v>
+      </c>
+      <c r="M28" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1800,12 +1886,15 @@
       <c r="K29" t="n">
         <v>0.00392368046067105</v>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L29" t="n">
+        <v>0.0997315494235569</v>
+      </c>
+      <c r="M29" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1847,12 +1936,15 @@
       <c r="K30" t="n">
         <v>-0.0007128893230051735</v>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L30" t="n">
+        <v>-0.01947460868452352</v>
+      </c>
+      <c r="M30" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1894,12 +1986,15 @@
       <c r="K31" t="n">
         <v>0.005059640365639088</v>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L31" t="n">
+        <v>0.1403327395698328</v>
+      </c>
+      <c r="M31" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1941,12 +2036,15 @@
       <c r="K32" t="n">
         <v>0.02271264005016667</v>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L32" t="n">
+        <v>0.7075798541342952</v>
+      </c>
+      <c r="M32" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -1988,12 +2086,15 @@
       <c r="K33" t="n">
         <v>0.03930504216182691</v>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L33" t="n">
+        <v>1.187152648437751</v>
+      </c>
+      <c r="M33" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>BR03_T_30</t>
         </is>
@@ -2035,12 +2136,15 @@
       <c r="K34" t="n">
         <v>0</v>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2082,12 +2186,15 @@
       <c r="K35" t="n">
         <v>0</v>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2129,12 +2236,15 @@
       <c r="K36" t="n">
         <v>0</v>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2176,12 +2286,15 @@
       <c r="K37" t="n">
         <v>0</v>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2223,12 +2336,15 @@
       <c r="K38" t="n">
         <v>0</v>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2270,12 +2386,15 @@
       <c r="K39" t="n">
         <v>0</v>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2317,12 +2436,15 @@
       <c r="K40" t="n">
         <v>0</v>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2364,12 +2486,15 @@
       <c r="K41" t="n">
         <v>0</v>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2411,12 +2536,15 @@
       <c r="K42" t="n">
         <v>0</v>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2458,12 +2586,15 @@
       <c r="K43" t="n">
         <v>0</v>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2505,12 +2636,15 @@
       <c r="K44" t="n">
         <v>0</v>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2552,12 +2686,15 @@
       <c r="K45" t="n">
         <v>0</v>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2599,12 +2736,15 @@
       <c r="K46" t="n">
         <v>0</v>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="N46" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2646,12 +2786,15 @@
       <c r="K47" t="n">
         <v>0</v>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="N47" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2693,12 +2836,15 @@
       <c r="K48" t="n">
         <v>0</v>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="N48" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2740,12 +2886,15 @@
       <c r="K49" t="n">
         <v>0.003501440435677357</v>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L49" t="n">
+        <v>0.1075442419529475</v>
+      </c>
+      <c r="M49" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="N49" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2787,12 +2936,15 @@
       <c r="K50" t="n">
         <v>0.001247265780681729</v>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L50" t="n">
+        <v>0.03939578058696151</v>
+      </c>
+      <c r="M50" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
+      <c r="N50" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2834,12 +2986,15 @@
       <c r="K51" t="n">
         <v>0.0005617989587166143</v>
       </c>
-      <c r="L51" t="inlineStr">
+      <c r="L51" t="n">
+        <v>0.01851729496427017</v>
+      </c>
+      <c r="M51" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
+      <c r="N51" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2881,12 +3036,15 @@
       <c r="K52" t="n">
         <v>0.001400303515493451</v>
       </c>
-      <c r="L52" t="inlineStr">
+      <c r="L52" t="n">
+        <v>0.04699852025274646</v>
+      </c>
+      <c r="M52" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
+      <c r="N52" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2928,12 +3086,15 @@
       <c r="K53" t="n">
         <v>0.002695343258845363</v>
       </c>
-      <c r="L53" t="inlineStr">
+      <c r="L53" t="n">
+        <v>0.09001483861951044</v>
+      </c>
+      <c r="M53" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="N53" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -2975,12 +3136,15 @@
       <c r="K54" t="n">
         <v>0.003184053625464791</v>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="L54" t="n">
+        <v>0.1083146813662575</v>
+      </c>
+      <c r="M54" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="N54" t="inlineStr">
         <is>
           <t>BR04_T_33</t>
         </is>
@@ -3022,12 +3186,15 @@
       <c r="K55" t="n">
         <v>0</v>
       </c>
-      <c r="L55" t="inlineStr">
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="N55" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3069,12 +3236,15 @@
       <c r="K56" t="n">
         <v>0</v>
       </c>
-      <c r="L56" t="inlineStr">
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
+      <c r="N56" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3116,12 +3286,15 @@
       <c r="K57" t="n">
         <v>0</v>
       </c>
-      <c r="L57" t="inlineStr">
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
+      <c r="N57" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3163,12 +3336,15 @@
       <c r="K58" t="n">
         <v>0</v>
       </c>
-      <c r="L58" t="inlineStr">
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
+      <c r="N58" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3210,12 +3386,15 @@
       <c r="K59" t="n">
         <v>0</v>
       </c>
-      <c r="L59" t="inlineStr">
+      <c r="L59" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr">
+      <c r="N59" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3257,12 +3436,15 @@
       <c r="K60" t="n">
         <v>0</v>
       </c>
-      <c r="L60" t="inlineStr">
+      <c r="L60" t="n">
+        <v>0</v>
+      </c>
+      <c r="M60" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr">
+      <c r="N60" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3304,12 +3486,15 @@
       <c r="K61" t="n">
         <v>0</v>
       </c>
-      <c r="L61" t="inlineStr">
+      <c r="L61" t="n">
+        <v>0</v>
+      </c>
+      <c r="M61" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr">
+      <c r="N61" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3351,12 +3536,15 @@
       <c r="K62" t="n">
         <v>0</v>
       </c>
-      <c r="L62" t="inlineStr">
+      <c r="L62" t="n">
+        <v>0</v>
+      </c>
+      <c r="M62" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
+      <c r="N62" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3398,12 +3586,15 @@
       <c r="K63" t="n">
         <v>0</v>
       </c>
-      <c r="L63" t="inlineStr">
+      <c r="L63" t="n">
+        <v>0</v>
+      </c>
+      <c r="M63" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="N63" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3445,12 +3636,15 @@
       <c r="K64" t="n">
         <v>0</v>
       </c>
-      <c r="L64" t="inlineStr">
+      <c r="L64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M64" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr">
+      <c r="N64" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3492,12 +3686,15 @@
       <c r="K65" t="n">
         <v>0</v>
       </c>
-      <c r="L65" t="inlineStr">
+      <c r="L65" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr">
+      <c r="N65" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3539,12 +3736,15 @@
       <c r="K66" t="n">
         <v>0</v>
       </c>
-      <c r="L66" t="inlineStr">
+      <c r="L66" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr">
+      <c r="N66" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3586,12 +3786,15 @@
       <c r="K67" t="n">
         <v>0</v>
       </c>
-      <c r="L67" t="inlineStr">
+      <c r="L67" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
+      <c r="N67" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3633,12 +3836,15 @@
       <c r="K68" t="n">
         <v>0</v>
       </c>
-      <c r="L68" t="inlineStr">
+      <c r="L68" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
+      <c r="N68" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3680,12 +3886,15 @@
       <c r="K69" t="n">
         <v>0</v>
       </c>
-      <c r="L69" t="inlineStr">
+      <c r="L69" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr">
+      <c r="N69" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3727,12 +3936,15 @@
       <c r="K70" t="n">
         <v>0.002547837117342036</v>
       </c>
-      <c r="L70" t="inlineStr">
+      <c r="L70" t="n">
+        <v>0.07468802521122649</v>
+      </c>
+      <c r="M70" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr">
+      <c r="N70" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3774,12 +3986,15 @@
       <c r="K71" t="n">
         <v>0.001724202920283548</v>
       </c>
-      <c r="L71" t="inlineStr">
+      <c r="L71" t="n">
+        <v>0.05183692922481049</v>
+      </c>
+      <c r="M71" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr">
+      <c r="N71" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3821,12 +4036,15 @@
       <c r="K72" t="n">
         <v>0.001413804742196162</v>
       </c>
-      <c r="L72" t="inlineStr">
+      <c r="L72" t="n">
+        <v>0.04374042576213553</v>
+      </c>
+      <c r="M72" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr">
+      <c r="N72" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3868,12 +4086,15 @@
       <c r="K73" t="n">
         <v>0.0007937774562501765</v>
       </c>
-      <c r="L73" t="inlineStr">
+      <c r="L73" t="n">
+        <v>0.02501154965717825</v>
+      </c>
+      <c r="M73" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr">
+      <c r="N73" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3915,12 +4136,15 @@
       <c r="K74" t="n">
         <v>0.0003337613079274545</v>
       </c>
-      <c r="L74" t="inlineStr">
+      <c r="L74" t="n">
+        <v>0.01059096150334082</v>
+      </c>
+      <c r="M74" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr">
+      <c r="N74" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -3962,12 +4186,15 @@
       <c r="K75" t="n">
         <v>-4.864082110984936e-05</v>
       </c>
-      <c r="L75" t="inlineStr">
+      <c r="L75" t="n">
+        <v>-0.001616033375635327</v>
+      </c>
+      <c r="M75" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr">
+      <c r="N75" t="inlineStr">
         <is>
           <t>BR05_T_37</t>
         </is>
@@ -4009,12 +4236,15 @@
       <c r="K76" t="n">
         <v>0</v>
       </c>
-      <c r="L76" t="inlineStr">
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr">
+      <c r="N76" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4056,12 +4286,15 @@
       <c r="K77" t="n">
         <v>0</v>
       </c>
-      <c r="L77" t="inlineStr">
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr">
+      <c r="N77" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4103,12 +4336,15 @@
       <c r="K78" t="n">
         <v>0</v>
       </c>
-      <c r="L78" t="inlineStr">
+      <c r="L78" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr">
+      <c r="N78" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4150,12 +4386,15 @@
       <c r="K79" t="n">
         <v>0</v>
       </c>
-      <c r="L79" t="inlineStr">
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr">
+      <c r="N79" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4197,12 +4436,15 @@
       <c r="K80" t="n">
         <v>0</v>
       </c>
-      <c r="L80" t="inlineStr">
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr">
+      <c r="N80" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4244,12 +4486,15 @@
       <c r="K81" t="n">
         <v>0</v>
       </c>
-      <c r="L81" t="inlineStr">
+      <c r="L81" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr">
+      <c r="N81" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4291,12 +4536,15 @@
       <c r="K82" t="n">
         <v>0</v>
       </c>
-      <c r="L82" t="inlineStr">
+      <c r="L82" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr">
+      <c r="N82" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4338,12 +4586,15 @@
       <c r="K83" t="n">
         <v>0</v>
       </c>
-      <c r="L83" t="inlineStr">
+      <c r="L83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr">
+      <c r="N83" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4385,12 +4636,15 @@
       <c r="K84" t="n">
         <v>0</v>
       </c>
-      <c r="L84" t="inlineStr">
+      <c r="L84" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr">
+      <c r="N84" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4432,12 +4686,15 @@
       <c r="K85" t="n">
         <v>0</v>
       </c>
-      <c r="L85" t="inlineStr">
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr">
+      <c r="N85" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4479,12 +4736,15 @@
       <c r="K86" t="n">
         <v>0</v>
       </c>
-      <c r="L86" t="inlineStr">
+      <c r="L86" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr">
+      <c r="N86" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4526,12 +4786,15 @@
       <c r="K87" t="n">
         <v>0</v>
       </c>
-      <c r="L87" t="inlineStr">
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr">
+      <c r="N87" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4573,12 +4836,15 @@
       <c r="K88" t="n">
         <v>0.001445001091803178</v>
       </c>
-      <c r="L88" t="inlineStr">
+      <c r="L88" t="n">
+        <v>0.04508919478244414</v>
+      </c>
+      <c r="M88" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr">
+      <c r="N88" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4620,12 +4886,15 @@
       <c r="K89" t="n">
         <v>0.001115254858587295</v>
       </c>
-      <c r="L89" t="inlineStr">
+      <c r="L89" t="n">
+        <v>0.03544120618467762</v>
+      </c>
+      <c r="M89" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr">
+      <c r="N89" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4667,12 +4936,15 @@
       <c r="K90" t="n">
         <v>0.001381250583328814</v>
       </c>
-      <c r="L90" t="inlineStr">
+      <c r="L90" t="n">
+        <v>0.04487091180699601</v>
+      </c>
+      <c r="M90" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr">
+      <c r="N90" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4714,12 +4986,15 @@
       <c r="K91" t="n">
         <v>0.001627618614383601</v>
       </c>
-      <c r="L91" t="inlineStr">
+      <c r="L91" t="n">
+        <v>0.05363584626756251</v>
+      </c>
+      <c r="M91" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr">
+      <c r="N91" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4761,12 +5036,15 @@
       <c r="K92" t="n">
         <v>0.001472810368952698</v>
       </c>
-      <c r="L92" t="inlineStr">
+      <c r="L92" t="n">
+        <v>0.04968104976699366</v>
+      </c>
+      <c r="M92" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M92" t="inlineStr">
+      <c r="N92" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4808,12 +5086,15 @@
       <c r="K93" t="n">
         <v>0.001562397105294549</v>
       </c>
-      <c r="L93" t="inlineStr">
+      <c r="L93" t="n">
+        <v>0.05339492107344111</v>
+      </c>
+      <c r="M93" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr">
+      <c r="N93" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4855,12 +5136,15 @@
       <c r="K94" t="n">
         <v>0.001741902445938169</v>
       </c>
-      <c r="L94" t="inlineStr">
+      <c r="L94" t="n">
+        <v>0.06140828229948458</v>
+      </c>
+      <c r="M94" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr">
+      <c r="N94" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4902,12 +5186,15 @@
       <c r="K95" t="n">
         <v>0.00157908576545168</v>
       </c>
-      <c r="L95" t="inlineStr">
+      <c r="L95" t="n">
+        <v>0.05786785371178452</v>
+      </c>
+      <c r="M95" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr">
+      <c r="N95" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4949,12 +5236,15 @@
       <c r="K96" t="n">
         <v>0.001512631426857109</v>
       </c>
-      <c r="L96" t="inlineStr">
+      <c r="L96" t="n">
+        <v>0.05670747174185383</v>
+      </c>
+      <c r="M96" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr">
+      <c r="N96" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -4996,12 +5286,15 @@
       <c r="K97" t="n">
         <v>0.001631883077251543</v>
       </c>
-      <c r="L97" t="inlineStr">
+      <c r="L97" t="n">
+        <v>0.06227382385868842</v>
+      </c>
+      <c r="M97" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr">
+      <c r="N97" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -5043,12 +5336,15 @@
       <c r="K98" t="n">
         <v>0.001589163588687227</v>
       </c>
-      <c r="L98" t="inlineStr">
+      <c r="L98" t="n">
+        <v>0.06114306907474112</v>
+      </c>
+      <c r="M98" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr">
+      <c r="N98" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -5090,12 +5386,15 @@
       <c r="K99" t="n">
         <v>0.001354066490569085</v>
       </c>
-      <c r="L99" t="inlineStr">
+      <c r="L99" t="n">
+        <v>0.05135297165483254</v>
+      </c>
+      <c r="M99" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M99" t="inlineStr">
+      <c r="N99" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -5137,12 +5436,15 @@
       <c r="K100" t="n">
         <v>0.001096025468330356</v>
       </c>
-      <c r="L100" t="inlineStr">
+      <c r="L100" t="n">
+        <v>0.04222046679075438</v>
+      </c>
+      <c r="M100" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M100" t="inlineStr">
+      <c r="N100" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -5184,12 +5486,15 @@
       <c r="K101" t="n">
         <v>0.0009206718114117425</v>
       </c>
-      <c r="L101" t="inlineStr">
+      <c r="L101" t="n">
+        <v>0.03576152364612189</v>
+      </c>
+      <c r="M101" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M101" t="inlineStr">
+      <c r="N101" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -5231,12 +5536,15 @@
       <c r="K102" t="n">
         <v>0.0006771604428841338</v>
       </c>
-      <c r="L102" t="inlineStr">
+      <c r="L102" t="n">
+        <v>0.02601021629721022</v>
+      </c>
+      <c r="M102" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M102" t="inlineStr">
+      <c r="N102" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -5278,12 +5586,15 @@
       <c r="K103" t="n">
         <v>-0.0002836589519597477</v>
       </c>
-      <c r="L103" t="inlineStr">
+      <c r="L103" t="n">
+        <v>-0.01084387650634693</v>
+      </c>
+      <c r="M103" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M103" t="inlineStr">
+      <c r="N103" t="inlineStr">
         <is>
           <t>BR06_T_29</t>
         </is>
@@ -5325,12 +5636,15 @@
       <c r="K104" t="n">
         <v>0</v>
       </c>
-      <c r="L104" t="inlineStr">
+      <c r="L104" t="n">
+        <v>0</v>
+      </c>
+      <c r="M104" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M104" t="inlineStr">
+      <c r="N104" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5372,12 +5686,15 @@
       <c r="K105" t="n">
         <v>0</v>
       </c>
-      <c r="L105" t="inlineStr">
+      <c r="L105" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M105" t="inlineStr">
+      <c r="N105" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5419,12 +5736,15 @@
       <c r="K106" t="n">
         <v>0</v>
       </c>
-      <c r="L106" t="inlineStr">
+      <c r="L106" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M106" t="inlineStr">
+      <c r="N106" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5466,12 +5786,15 @@
       <c r="K107" t="n">
         <v>0</v>
       </c>
-      <c r="L107" t="inlineStr">
+      <c r="L107" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M107" t="inlineStr">
+      <c r="N107" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5513,12 +5836,15 @@
       <c r="K108" t="n">
         <v>0</v>
       </c>
-      <c r="L108" t="inlineStr">
+      <c r="L108" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr">
+      <c r="N108" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5560,12 +5886,15 @@
       <c r="K109" t="n">
         <v>0</v>
       </c>
-      <c r="L109" t="inlineStr">
+      <c r="L109" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr">
+      <c r="N109" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5607,12 +5936,15 @@
       <c r="K110" t="n">
         <v>0</v>
       </c>
-      <c r="L110" t="inlineStr">
+      <c r="L110" t="n">
+        <v>0</v>
+      </c>
+      <c r="M110" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr">
+      <c r="N110" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5654,12 +5986,15 @@
       <c r="K111" t="n">
         <v>0</v>
       </c>
-      <c r="L111" t="inlineStr">
+      <c r="L111" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M111" t="inlineStr">
+      <c r="N111" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5701,12 +6036,15 @@
       <c r="K112" t="n">
         <v>0</v>
       </c>
-      <c r="L112" t="inlineStr">
+      <c r="L112" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M112" t="inlineStr">
+      <c r="N112" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5748,12 +6086,15 @@
       <c r="K113" t="n">
         <v>0</v>
       </c>
-      <c r="L113" t="inlineStr">
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
+      <c r="M113" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M113" t="inlineStr">
+      <c r="N113" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5795,12 +6136,15 @@
       <c r="K114" t="n">
         <v>0</v>
       </c>
-      <c r="L114" t="inlineStr">
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
+      <c r="M114" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M114" t="inlineStr">
+      <c r="N114" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5842,12 +6186,15 @@
       <c r="K115" t="n">
         <v>0.0001175005555978089</v>
       </c>
-      <c r="L115" t="inlineStr">
+      <c r="L115" t="n">
+        <v>0.002487234975100769</v>
+      </c>
+      <c r="M115" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M115" t="inlineStr">
+      <c r="N115" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5889,12 +6236,15 @@
       <c r="K116" t="n">
         <v>-0.0004264984994682457</v>
       </c>
-      <c r="L116" t="inlineStr">
+      <c r="L116" t="n">
+        <v>-0.009958739962583571</v>
+      </c>
+      <c r="M116" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M116" t="inlineStr">
+      <c r="N116" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5936,12 +6286,15 @@
       <c r="K117" t="n">
         <v>0.00164594032461177</v>
       </c>
-      <c r="L117" t="inlineStr">
+      <c r="L117" t="n">
+        <v>0.04138952080568374</v>
+      </c>
+      <c r="M117" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M117" t="inlineStr">
+      <c r="N117" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -5983,12 +6336,15 @@
       <c r="K118" t="n">
         <v>0.003312583250983506</v>
       </c>
-      <c r="L118" t="inlineStr">
+      <c r="L118" t="n">
+        <v>0.0836072351239299</v>
+      </c>
+      <c r="M118" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr">
+      <c r="N118" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6030,12 +6386,15 @@
       <c r="K119" t="n">
         <v>0.002739171059580418</v>
       </c>
-      <c r="L119" t="inlineStr">
+      <c r="L119" t="n">
+        <v>0.0658477157215564</v>
+      </c>
+      <c r="M119" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr">
+      <c r="N119" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6077,12 +6436,15 @@
       <c r="K120" t="n">
         <v>0.001911362494183918</v>
       </c>
-      <c r="L120" t="inlineStr">
+      <c r="L120" t="n">
+        <v>0.04783867271157457</v>
+      </c>
+      <c r="M120" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M120" t="inlineStr">
+      <c r="N120" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6124,12 +6486,15 @@
       <c r="K121" t="n">
         <v>0.001315088996618529</v>
       </c>
-      <c r="L121" t="inlineStr">
+      <c r="L121" t="n">
+        <v>0.03453047965406929</v>
+      </c>
+      <c r="M121" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M121" t="inlineStr">
+      <c r="N121" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6171,12 +6536,15 @@
       <c r="K122" t="n">
         <v>5.015906025550427e-05</v>
       </c>
-      <c r="L122" t="inlineStr">
+      <c r="L122" t="n">
+        <v>0.001374358251000819</v>
+      </c>
+      <c r="M122" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M122" t="inlineStr">
+      <c r="N122" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6218,12 +6586,15 @@
       <c r="K123" t="n">
         <v>-0.0001059684095731</v>
       </c>
-      <c r="L123" t="inlineStr">
+      <c r="L123" t="n">
+        <v>-0.003015936628171551</v>
+      </c>
+      <c r="M123" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M123" t="inlineStr">
+      <c r="N123" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6265,12 +6636,15 @@
       <c r="K124" t="n">
         <v>-0.0001650741561724392</v>
       </c>
-      <c r="L124" t="inlineStr">
+      <c r="L124" t="n">
+        <v>-0.004734680529360216</v>
+      </c>
+      <c r="M124" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M124" t="inlineStr">
+      <c r="N124" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6312,12 +6686,15 @@
       <c r="K125" t="n">
         <v>-0.0002678445384691147</v>
       </c>
-      <c r="L125" t="inlineStr">
+      <c r="L125" t="n">
+        <v>-0.007710096357360944</v>
+      </c>
+      <c r="M125" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M125" t="inlineStr">
+      <c r="N125" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6359,12 +6736,15 @@
       <c r="K126" t="n">
         <v>-0.0001556484430730202</v>
       </c>
-      <c r="L126" t="inlineStr">
+      <c r="L126" t="n">
+        <v>-0.004483231047799664</v>
+      </c>
+      <c r="M126" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M126" t="inlineStr">
+      <c r="N126" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6406,12 +6786,15 @@
       <c r="K127" t="n">
         <v>-1.403233585153209e-05</v>
       </c>
-      <c r="L127" t="inlineStr">
+      <c r="L127" t="n">
+        <v>-0.0004181636083756561</v>
+      </c>
+      <c r="M127" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M127" t="inlineStr">
+      <c r="N127" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6453,12 +6836,15 @@
       <c r="K128" t="n">
         <v>0.000295096461983429</v>
       </c>
-      <c r="L128" t="inlineStr">
+      <c r="L128" t="n">
+        <v>0.009184877379234234</v>
+      </c>
+      <c r="M128" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M128" t="inlineStr">
+      <c r="N128" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6500,12 +6886,15 @@
       <c r="K129" t="n">
         <v>0.0006443471915813714</v>
       </c>
-      <c r="L129" t="inlineStr">
+      <c r="L129" t="n">
+        <v>0.01989882202001472</v>
+      </c>
+      <c r="M129" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M129" t="inlineStr">
+      <c r="N129" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6547,12 +6936,15 @@
       <c r="K130" t="n">
         <v>0.002583354190690231</v>
       </c>
-      <c r="L130" t="inlineStr">
+      <c r="L130" t="n">
+        <v>0.08250126133268612</v>
+      </c>
+      <c r="M130" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="M130" t="inlineStr">
+      <c r="N130" t="inlineStr">
         <is>
           <t>BR07_T_32</t>
         </is>
@@ -6594,12 +6986,15 @@
       <c r="K131" t="n">
         <v>0</v>
       </c>
-      <c r="L131" t="inlineStr">
+      <c r="L131" t="n">
+        <v>0</v>
+      </c>
+      <c r="M131" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M131" t="inlineStr">
+      <c r="N131" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -6641,12 +7036,15 @@
       <c r="K132" t="n">
         <v>0</v>
       </c>
-      <c r="L132" t="inlineStr">
+      <c r="L132" t="n">
+        <v>0</v>
+      </c>
+      <c r="M132" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr">
+      <c r="N132" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -6688,12 +7086,15 @@
       <c r="K133" t="n">
         <v>0</v>
       </c>
-      <c r="L133" t="inlineStr">
+      <c r="L133" t="n">
+        <v>0</v>
+      </c>
+      <c r="M133" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
+      <c r="N133" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -6735,12 +7136,15 @@
       <c r="K134" t="n">
         <v>0</v>
       </c>
-      <c r="L134" t="inlineStr">
+      <c r="L134" t="n">
+        <v>0</v>
+      </c>
+      <c r="M134" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr">
+      <c r="N134" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -6782,12 +7186,15 @@
       <c r="K135" t="n">
         <v>0</v>
       </c>
-      <c r="L135" t="inlineStr">
+      <c r="L135" t="n">
+        <v>0</v>
+      </c>
+      <c r="M135" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M135" t="inlineStr">
+      <c r="N135" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -6829,12 +7236,15 @@
       <c r="K136" t="n">
         <v>0</v>
       </c>
-      <c r="L136" t="inlineStr">
+      <c r="L136" t="n">
+        <v>0</v>
+      </c>
+      <c r="M136" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M136" t="inlineStr">
+      <c r="N136" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -6876,12 +7286,15 @@
       <c r="K137" t="n">
         <v>0</v>
       </c>
-      <c r="L137" t="inlineStr">
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M137" t="inlineStr">
+      <c r="N137" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -6923,12 +7336,15 @@
       <c r="K138" t="n">
         <v>0</v>
       </c>
-      <c r="L138" t="inlineStr">
+      <c r="L138" t="n">
+        <v>0</v>
+      </c>
+      <c r="M138" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M138" t="inlineStr">
+      <c r="N138" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -6970,12 +7386,15 @@
       <c r="K139" t="n">
         <v>0</v>
       </c>
-      <c r="L139" t="inlineStr">
+      <c r="L139" t="n">
+        <v>0</v>
+      </c>
+      <c r="M139" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M139" t="inlineStr">
+      <c r="N139" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7017,12 +7436,15 @@
       <c r="K140" t="n">
         <v>0</v>
       </c>
-      <c r="L140" t="inlineStr">
+      <c r="L140" t="n">
+        <v>0</v>
+      </c>
+      <c r="M140" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M140" t="inlineStr">
+      <c r="N140" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7064,12 +7486,15 @@
       <c r="K141" t="n">
         <v>0</v>
       </c>
-      <c r="L141" t="inlineStr">
+      <c r="L141" t="n">
+        <v>0</v>
+      </c>
+      <c r="M141" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M141" t="inlineStr">
+      <c r="N141" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7111,12 +7536,15 @@
       <c r="K142" t="n">
         <v>0.001811100575128213</v>
       </c>
-      <c r="L142" t="inlineStr">
+      <c r="L142" t="n">
+        <v>0.05035506420490406</v>
+      </c>
+      <c r="M142" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M142" t="inlineStr">
+      <c r="N142" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7158,12 +7586,15 @@
       <c r="K143" t="n">
         <v>0.001329836581426537</v>
       </c>
-      <c r="L143" t="inlineStr">
+      <c r="L143" t="n">
+        <v>0.03751563984531511</v>
+      </c>
+      <c r="M143" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M143" t="inlineStr">
+      <c r="N143" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7205,12 +7636,15 @@
       <c r="K144" t="n">
         <v>0.001320393462500107</v>
       </c>
-      <c r="L144" t="inlineStr">
+      <c r="L144" t="n">
+        <v>0.03809335139312801</v>
+      </c>
+      <c r="M144" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M144" t="inlineStr">
+      <c r="N144" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7252,12 +7686,15 @@
       <c r="K145" t="n">
         <v>0.0008079556498792349</v>
       </c>
-      <c r="L145" t="inlineStr">
+      <c r="L145" t="n">
+        <v>0.02409439170175586</v>
+      </c>
+      <c r="M145" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M145" t="inlineStr">
+      <c r="N145" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7299,12 +7736,15 @@
       <c r="K146" t="n">
         <v>0.0005147638662777166</v>
       </c>
-      <c r="L146" t="inlineStr">
+      <c r="L146" t="n">
+        <v>0.01553851499206882</v>
+      </c>
+      <c r="M146" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M146" t="inlineStr">
+      <c r="N146" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7346,12 +7786,15 @@
       <c r="K147" t="n">
         <v>8.924070142373759e-05</v>
       </c>
-      <c r="L147" t="inlineStr">
+      <c r="L147" t="n">
+        <v>0.002899366645899068</v>
+      </c>
+      <c r="M147" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M147" t="inlineStr">
+      <c r="N147" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7393,12 +7836,15 @@
       <c r="K148" t="n">
         <v>7.319109800795945e-05</v>
       </c>
-      <c r="L148" t="inlineStr">
+      <c r="L148" t="n">
+        <v>0.002410339695469268</v>
+      </c>
+      <c r="M148" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M148" t="inlineStr">
+      <c r="N148" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7440,12 +7886,15 @@
       <c r="K149" t="n">
         <v>8.366395206795795e-05</v>
       </c>
-      <c r="L149" t="inlineStr">
+      <c r="L149" t="n">
+        <v>0.002780631206944343</v>
+      </c>
+      <c r="M149" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M149" t="inlineStr">
+      <c r="N149" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7487,12 +7936,15 @@
       <c r="K150" t="n">
         <v>9.984344484120283e-05</v>
       </c>
-      <c r="L150" t="inlineStr">
+      <c r="L150" t="n">
+        <v>0.003288415172591337</v>
+      </c>
+      <c r="M150" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M150" t="inlineStr">
+      <c r="N150" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7534,12 +7986,15 @@
       <c r="K151" t="n">
         <v>0.0001854793019686192</v>
       </c>
-      <c r="L151" t="inlineStr">
+      <c r="L151" t="n">
+        <v>0.006477864621254031</v>
+      </c>
+      <c r="M151" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M151" t="inlineStr">
+      <c r="N151" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7581,12 +8036,15 @@
       <c r="K152" t="n">
         <v>0.0003644512203400279</v>
       </c>
-      <c r="L152" t="inlineStr">
+      <c r="L152" t="n">
+        <v>0.01287423935851149</v>
+      </c>
+      <c r="M152" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M152" t="inlineStr">
+      <c r="N152" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7628,12 +8086,15 @@
       <c r="K153" t="n">
         <v>0.000570465953039973</v>
       </c>
-      <c r="L153" t="inlineStr">
+      <c r="L153" t="n">
+        <v>0.02094424999018182</v>
+      </c>
+      <c r="M153" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M153" t="inlineStr">
+      <c r="N153" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7675,12 +8136,15 @@
       <c r="K154" t="n">
         <v>0.0008263887538865186</v>
       </c>
-      <c r="L154" t="inlineStr">
+      <c r="L154" t="n">
+        <v>0.03020450895455222</v>
+      </c>
+      <c r="M154" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M154" t="inlineStr">
+      <c r="N154" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>
@@ -7722,12 +8186,15 @@
       <c r="K155" t="n">
         <v>0.001747875790330702</v>
       </c>
-      <c r="L155" t="inlineStr">
+      <c r="L155" t="n">
+        <v>0.06546419076142171</v>
+      </c>
+      <c r="M155" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="M155" t="inlineStr">
+      <c r="N155" t="inlineStr">
         <is>
           <t>BR08_T_29</t>
         </is>

</xml_diff>